<commit_message>
CMDB §15 governance haircut set at 30% (owner decision, TEN-equivalent)
Owner sized the haircut at 30% citing TEN-equivalence: management
concerns, related-party transactions ($21.6M/yr fees to
Costamare-affiliated managers), and lack of return to common (no
dividend/buyback despite net cash), plus family control and the
persistent 0.6x P/BV print.

Mechanics: applied at the blend layer + strip terminal per S15
convention; asset NAV untouched at $32.23. With payout 0 the entire
strip is terminal NAV, so the haircut passes through ~1:1 - PW FV
$28.32 -> $19.82, EV +64.2% -> +14.9% (mild BUY vs price $17.25).
The -30% FV drift flag is the haircut application, annotated.

S15.3 gains its second-case entry (no external anchor to triangulate
the 30%, unlike TEN's VIE cross-check - it is a TEN-equivalence
judgment; revisit trigger = any payout initiation). CLAUDE.md
quick-ref + changelog updated.

tests: 210 passed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -563,7 +563,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CMDB</t>
+          <t>STNG</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -572,23 +572,23 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.62</v>
+        <v>0.7</v>
       </c>
       <c r="D3" t="n">
-        <v>0.843</v>
+        <v>1.373</v>
       </c>
       <c r="E3" t="n">
-        <v>64.2</v>
+        <v>-3.3</v>
       </c>
       <c r="F3" t="n">
-        <v>53</v>
+        <v>13.1</v>
       </c>
       <c r="G3" t="n">
-        <v>41.9</v>
+        <v>29.4</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>BUY (undervalued)</t>
+          <t>HOLD (fairly valued)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -597,25 +597,25 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>2725019</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>28.32</v>
+        <v>73.13</v>
       </c>
       <c r="M3" t="n">
-        <v>24.47</v>
+        <v>97.81999999999999</v>
       </c>
       <c r="N3" t="n">
-        <v>-22.3</v>
+        <v>32.7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>STNG</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -624,23 +624,23 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="D4" t="n">
-        <v>1.373</v>
+        <v>1.979</v>
       </c>
       <c r="E4" t="n">
-        <v>-3.3</v>
+        <v>-44.9</v>
       </c>
       <c r="F4" t="n">
-        <v>13.1</v>
+        <v>-8.9</v>
       </c>
       <c r="G4" t="n">
-        <v>29.4</v>
+        <v>27.2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>HOLD (fairly valued)</t>
+          <t>TRIM/SHORT (overvalued)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -649,25 +649,25 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2725019</v>
+        <v>334239</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>73.13</v>
+        <v>2.86</v>
       </c>
       <c r="M4" t="n">
-        <v>97.81999999999999</v>
+        <v>6.61</v>
       </c>
       <c r="N4" t="n">
-        <v>32.7</v>
+        <v>72.09999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>ASC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -676,19 +676,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.85</v>
+        <v>0.75</v>
       </c>
       <c r="D5" t="n">
-        <v>1.979</v>
+        <v>1.331</v>
       </c>
       <c r="E5" t="n">
-        <v>-44.9</v>
+        <v>-5.9</v>
       </c>
       <c r="F5" t="n">
-        <v>-8.9</v>
+        <v>9.1</v>
       </c>
       <c r="G5" t="n">
-        <v>27.2</v>
+        <v>24.2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -701,25 +701,25 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>334239</v>
+        <v>38532</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>2.86</v>
+        <v>15.05</v>
       </c>
       <c r="M5" t="n">
-        <v>6.61</v>
+        <v>19.87</v>
       </c>
       <c r="N5" t="n">
-        <v>72.09999999999999</v>
+        <v>30.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASC</t>
+          <t>TNK</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -728,23 +728,23 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="D6" t="n">
-        <v>1.331</v>
+        <v>1.342</v>
       </c>
       <c r="E6" t="n">
-        <v>-5.9</v>
+        <v>4.1</v>
       </c>
       <c r="F6" t="n">
-        <v>9.1</v>
+        <v>14</v>
       </c>
       <c r="G6" t="n">
-        <v>24.2</v>
+        <v>23.9</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>TRIM/SHORT (overvalued)</t>
+          <t>HOLD (fairly valued)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -753,25 +753,25 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>38532</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>15.05</v>
+        <v>73.7</v>
       </c>
       <c r="M6" t="n">
-        <v>19.87</v>
+        <v>87.73</v>
       </c>
       <c r="N6" t="n">
-        <v>30.1</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TNK</t>
+          <t>TRMD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -780,23 +780,23 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.76</v>
+        <v>0.83</v>
       </c>
       <c r="D7" t="n">
-        <v>1.342</v>
+        <v>1.237</v>
       </c>
       <c r="E7" t="n">
-        <v>4.1</v>
+        <v>-5.4</v>
       </c>
       <c r="F7" t="n">
-        <v>14</v>
+        <v>8.1</v>
       </c>
       <c r="G7" t="n">
-        <v>23.9</v>
+        <v>21.7</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>HOLD (fairly valued)</t>
+          <t>TRIM/SHORT (overvalued)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -805,25 +805,25 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>68988</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>73.7</v>
+        <v>26.68</v>
       </c>
       <c r="M7" t="n">
-        <v>87.73</v>
+        <v>34.31</v>
       </c>
       <c r="N7" t="n">
-        <v>19.8</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TRMD</t>
+          <t>CCEC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -832,23 +832,23 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.83</v>
+        <v>0.9</v>
       </c>
       <c r="D8" t="n">
-        <v>1.237</v>
+        <v>0.962</v>
       </c>
       <c r="E8" t="n">
-        <v>-5.4</v>
+        <v>35.3</v>
       </c>
       <c r="F8" t="n">
-        <v>8.1</v>
+        <v>27.3</v>
       </c>
       <c r="G8" t="n">
-        <v>21.7</v>
+        <v>19.2</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>TRIM/SHORT (overvalued)</t>
+          <t>BUY (undervalued)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -857,25 +857,25 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>68988</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>2977992</v>
       </c>
       <c r="L8" t="n">
-        <v>26.68</v>
+        <v>29.63</v>
       </c>
       <c r="M8" t="n">
-        <v>34.31</v>
+        <v>26.11</v>
       </c>
       <c r="N8" t="n">
-        <v>27.1</v>
+        <v>-16.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CCEC</t>
+          <t>SBLK</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -884,23 +884,23 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.9</v>
+        <v>0.82</v>
       </c>
       <c r="D9" t="n">
-        <v>0.962</v>
+        <v>1.211</v>
       </c>
       <c r="E9" t="n">
-        <v>35.3</v>
+        <v>-5.4</v>
       </c>
       <c r="F9" t="n">
-        <v>27.3</v>
+        <v>5.7</v>
       </c>
       <c r="G9" t="n">
-        <v>19.2</v>
+        <v>16.8</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>BUY (undervalued)</t>
+          <t>TRIM/SHORT (overvalued)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="J9" t="n">
+        <v>28583</v>
+      </c>
+      <c r="K9" t="n">
         <v>0</v>
       </c>
-      <c r="K9" t="n">
-        <v>2977992</v>
-      </c>
       <c r="L9" t="n">
-        <v>29.63</v>
+        <v>25.72</v>
       </c>
       <c r="M9" t="n">
-        <v>26.11</v>
+        <v>31.77</v>
       </c>
       <c r="N9" t="n">
-        <v>-16.1</v>
+        <v>22.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SBLK</t>
+          <t>GNK</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -936,23 +936,23 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.82</v>
+        <v>0.87</v>
       </c>
       <c r="D10" t="n">
-        <v>1.211</v>
+        <v>1.042</v>
       </c>
       <c r="E10" t="n">
-        <v>-5.4</v>
+        <v>7.2</v>
       </c>
       <c r="F10" t="n">
-        <v>5.7</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>16.8</v>
+        <v>12.1</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>TRIM/SHORT (overvalued)</t>
+          <t>BUY (undervalued)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -961,50 +961,50 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>28583</v>
+        <v>18314</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>12474</v>
       </c>
       <c r="L10" t="n">
-        <v>25.72</v>
+        <v>25.73</v>
       </c>
       <c r="M10" t="n">
-        <v>31.77</v>
+        <v>26.91</v>
       </c>
       <c r="N10" t="n">
-        <v>22.3</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GNK</t>
+          <t>INSW</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>whole-company</t>
+          <t>WHOLE-COMPANY (hybrid aggregation)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.87</v>
+        <v>0.98</v>
       </c>
       <c r="D11" t="n">
-        <v>1.042</v>
+        <v>1.518</v>
       </c>
       <c r="E11" t="n">
-        <v>7.2</v>
+        <v>-23.8</v>
       </c>
       <c r="F11" t="n">
+        <v>-7</v>
+      </c>
+      <c r="G11" t="n">
         <v>9.699999999999999</v>
       </c>
-      <c r="G11" t="n">
-        <v>12.1</v>
-      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>BUY (undervalued)</t>
+          <t>TRIM/SHORT (overvalued)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1013,46 +1013,46 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>18314</v>
+        <v>342121</v>
       </c>
       <c r="K11" t="n">
-        <v>12474</v>
+        <v>67887</v>
       </c>
       <c r="L11" t="n">
-        <v>25.73</v>
+        <v>59.47</v>
       </c>
       <c r="M11" t="n">
-        <v>26.91</v>
+        <v>85.54000000000001</v>
       </c>
       <c r="N11" t="n">
-        <v>4.9</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>INSW</t>
+          <t>HAFN</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>WHOLE-COMPANY (hybrid aggregation)</t>
+          <t>whole-company</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="D12" t="n">
-        <v>1.518</v>
+        <v>1.433</v>
       </c>
       <c r="E12" t="n">
-        <v>-23.8</v>
+        <v>-25.1</v>
       </c>
       <c r="F12" t="n">
-        <v>-7</v>
+        <v>-8.4</v>
       </c>
       <c r="G12" t="n">
-        <v>9.699999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1065,16 +1065,16 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>342121</v>
+        <v>126273</v>
       </c>
       <c r="K12" t="n">
-        <v>67887</v>
+        <v>28673</v>
       </c>
       <c r="L12" t="n">
-        <v>59.47</v>
+        <v>5.77</v>
       </c>
       <c r="M12" t="n">
-        <v>85.54000000000001</v>
+        <v>8.34</v>
       </c>
       <c r="N12" t="n">
         <v>33.4</v>
@@ -1083,7 +1083,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HAFN</t>
+          <t>DHT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1092,19 +1092,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.95</v>
+        <v>1.09</v>
       </c>
       <c r="D13" t="n">
-        <v>1.433</v>
+        <v>1.145</v>
       </c>
       <c r="E13" t="n">
-        <v>-25.1</v>
+        <v>-8.1</v>
       </c>
       <c r="F13" t="n">
-        <v>-8.4</v>
+        <v>-2</v>
       </c>
       <c r="G13" t="n">
-        <v>8.300000000000001</v>
+        <v>4</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1113,29 +1113,29 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>BUY (undervalued)</t>
+          <t>HOLD (fairly valued)</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>126273</v>
+        <v>315444</v>
       </c>
       <c r="K13" t="n">
-        <v>28673</v>
+        <v>168393</v>
       </c>
       <c r="L13" t="n">
-        <v>5.77</v>
+        <v>15.08</v>
       </c>
       <c r="M13" t="n">
-        <v>8.34</v>
+        <v>17.05</v>
       </c>
       <c r="N13" t="n">
-        <v>33.4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DHT</t>
+          <t>CMDB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1144,23 +1144,23 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1.09</v>
+        <v>0.62</v>
       </c>
       <c r="D14" t="n">
-        <v>1.145</v>
+        <v>0.843</v>
       </c>
       <c r="E14" t="n">
-        <v>-8.1</v>
+        <v>14.9</v>
       </c>
       <c r="F14" t="n">
-        <v>-2</v>
+        <v>7.1</v>
       </c>
       <c r="G14" t="n">
-        <v>4</v>
+        <v>-0.7</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>TRIM/SHORT (overvalued)</t>
+          <t>BUY (undervalued)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1169,19 +1169,19 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>315444</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>168393</v>
+        <v>1070509</v>
       </c>
       <c r="L14" t="n">
-        <v>15.08</v>
+        <v>19.82</v>
       </c>
       <c r="M14" t="n">
-        <v>17.05</v>
+        <v>17.13</v>
       </c>
       <c r="N14" t="n">
-        <v>12</v>
+        <v>-15.6</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
CAPT: refine §9.6 newbuild cohorts to exact Q1-release delivery dates
Replaced the rollout's estimated cohorts with per-vessel years_to_delivery from
CAPT's Q1 earnings release (from the Mar-31 snapshot): VLCC 1 delivered
(Aristotelis II) / 7 in 2027 / 4 in 2028; Suezmax NB 6 near-term 2026 / 2 in 2028.
NAV $15.05 -> $15.03 (-0.1pp, stable) — the estimate was already accurate, so a
precision/provenance upgrade, not a re-rate. CAPT -17.5% divergence + BUY stand.
286 tests green. Includes the pipeline-run artifacts (outputs + decision-log
stubs) to keep the tree clean.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -581,10 +581,10 @@
         <v>22.4</v>
       </c>
       <c r="F3" t="n">
-        <v>39.6</v>
+        <v>39.7</v>
       </c>
       <c r="G3" t="n">
-        <v>56.9</v>
+        <v>57.1</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -606,10 +606,10 @@
         <v>16.2</v>
       </c>
       <c r="M3" t="n">
-        <v>20.78</v>
+        <v>20.8</v>
       </c>
       <c r="N3" t="n">
-        <v>34.6</v>
+        <v>34.7</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
fix: BUG-1 Aframax dual cycle-anchor + BUG-2 Sinokor row in VLCC fit
BUG-1: historical_tce_means.yaml carried a stale Aframax 10yr-mean (27600) vs
scenario_inputs aframax_dirty (36483), so the per-name FV path and the scenario
path computed different cycle positions for every Aframax name. Reconciled to
36483 + test_cycle_anchor_cross_file_consistency guard.

BUG-2: the Sinokor en-bloc VLCC row (age 12, $71M, labeled documentation-only)
was actually in the regression - fit_curve_anchors filtered on age only. Added an
in_fit flag (TransactionPrint + loader + fit) and set in_fit:false on the two doc
rows. VLCC age-10 anchor rises -> VLCC NAVs +0.3-1.1pp, all under the 2pp drift
gate, SANITY 0 fail, no flips. Tests 290 -> 291.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -523,13 +523,13 @@
         <v>0.34</v>
       </c>
       <c r="D2" t="n">
-        <v>1.195</v>
+        <v>1.194</v>
       </c>
       <c r="E2" t="n">
-        <v>69.3</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>90.2</v>
+        <v>90.3</v>
       </c>
       <c r="G2" t="n">
         <v>111</v>
@@ -551,19 +551,19 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>64.84</v>
+        <v>64.93000000000001</v>
       </c>
       <c r="M2" t="n">
-        <v>80.79000000000001</v>
+        <v>80.8</v>
       </c>
       <c r="N2" t="n">
-        <v>41.7</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAPT</t>
+          <t>BRUT</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -572,16 +572,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.67</v>
+        <v>0.75</v>
       </c>
       <c r="D3" t="n">
-        <v>1.171</v>
+        <v>0.926</v>
       </c>
       <c r="E3" t="n">
-        <v>26.7</v>
+        <v>100.1</v>
       </c>
       <c r="F3" t="n">
-        <v>43.6</v>
+        <v>80.3</v>
       </c>
       <c r="G3" t="n">
         <v>60.5</v>
@@ -597,25 +597,25 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>2791</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>16.77</v>
+        <v>10.81</v>
       </c>
       <c r="M3" t="n">
-        <v>21.25</v>
+        <v>8.67</v>
       </c>
       <c r="N3" t="n">
-        <v>33.8</v>
+        <v>-39.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BRUT</t>
+          <t>CAPT</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -624,16 +624,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.75</v>
+        <v>0.67</v>
       </c>
       <c r="D4" t="n">
-        <v>0.926</v>
+        <v>1.171</v>
       </c>
       <c r="E4" t="n">
-        <v>100.1</v>
+        <v>26.7</v>
       </c>
       <c r="F4" t="n">
-        <v>80.3</v>
+        <v>43.6</v>
       </c>
       <c r="G4" t="n">
         <v>60.5</v>
@@ -649,19 +649,19 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>2701</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>10.8</v>
+        <v>16.77</v>
       </c>
       <c r="M4" t="n">
-        <v>8.67</v>
+        <v>21.25</v>
       </c>
       <c r="N4" t="n">
-        <v>-39.6</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="5">
@@ -835,7 +835,7 @@
         <v>0.76</v>
       </c>
       <c r="D8" t="n">
-        <v>1.446</v>
+        <v>1.445</v>
       </c>
       <c r="E8" t="n">
         <v>6.9</v>
@@ -857,19 +857,19 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>41889</v>
+        <v>41652</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>79.56</v>
+        <v>79.59</v>
       </c>
       <c r="M8" t="n">
-        <v>97.48</v>
+        <v>97.48999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>24.1</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -1199,13 +1199,13 @@
         <v>0.98</v>
       </c>
       <c r="D15" t="n">
-        <v>1.645</v>
+        <v>1.638</v>
       </c>
       <c r="E15" t="n">
-        <v>-27.6</v>
+        <v>-27.4</v>
       </c>
       <c r="F15" t="n">
-        <v>-8.800000000000001</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="G15" t="n">
         <v>9.9</v>
@@ -1221,19 +1221,19 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>316872</v>
+        <v>316781</v>
       </c>
       <c r="K15" t="n">
-        <v>74962</v>
+        <v>75231</v>
       </c>
       <c r="L15" t="n">
-        <v>61.16</v>
+        <v>61.34</v>
       </c>
       <c r="M15" t="n">
-        <v>92.90000000000001</v>
+        <v>92.89</v>
       </c>
       <c r="N15" t="n">
-        <v>37.6</v>
+        <v>37.3</v>
       </c>
     </row>
     <row r="16">
@@ -1303,16 +1303,16 @@
         <v>1.09</v>
       </c>
       <c r="D17" t="n">
-        <v>1.301</v>
+        <v>1.287</v>
       </c>
       <c r="E17" t="n">
-        <v>-21.8</v>
+        <v>-21</v>
       </c>
       <c r="F17" t="n">
-        <v>-11.2</v>
+        <v>-10.8</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.6</v>
+        <v>-0.5</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1325,19 +1325,19 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>529540</v>
+        <v>518123</v>
       </c>
       <c r="K17" t="n">
-        <v>230527</v>
+        <v>230052</v>
       </c>
       <c r="L17" t="n">
-        <v>14.77</v>
+        <v>14.92</v>
       </c>
       <c r="M17" t="n">
-        <v>18.78</v>
+        <v>18.79</v>
       </c>
       <c r="N17" t="n">
-        <v>21.3</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="18">
@@ -1407,16 +1407,16 @@
         <v>1.2</v>
       </c>
       <c r="D19" t="n">
-        <v>1.274</v>
+        <v>1.269</v>
       </c>
       <c r="E19" t="n">
-        <v>-29.9</v>
+        <v>-29.6</v>
       </c>
       <c r="F19" t="n">
-        <v>-18.6</v>
+        <v>-18.5</v>
       </c>
       <c r="G19" t="n">
-        <v>-7.4</v>
+        <v>-7.3</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1429,19 +1429,19 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>469143</v>
+        <v>466274</v>
       </c>
       <c r="K19" t="n">
-        <v>260767</v>
+        <v>260547</v>
       </c>
       <c r="L19" t="n">
-        <v>28.68</v>
+        <v>28.82</v>
       </c>
       <c r="M19" t="n">
-        <v>37.92</v>
+        <v>37.94</v>
       </c>
       <c r="N19" t="n">
-        <v>22.6</v>
+        <v>22.3</v>
       </c>
     </row>
     <row r="20">
@@ -1459,13 +1459,13 @@
         <v>1.21</v>
       </c>
       <c r="D20" t="n">
-        <v>1.199</v>
+        <v>1.195</v>
       </c>
       <c r="E20" t="n">
-        <v>-24.9</v>
+        <v>-24.6</v>
       </c>
       <c r="F20" t="n">
-        <v>-16.4</v>
+        <v>-16.2</v>
       </c>
       <c r="G20" t="n">
         <v>-7.9</v>
@@ -1481,19 +1481,19 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>343849</v>
+        <v>341712</v>
       </c>
       <c r="K20" t="n">
-        <v>222252</v>
+        <v>222060</v>
       </c>
       <c r="L20" t="n">
-        <v>39.41</v>
+        <v>39.59</v>
       </c>
       <c r="M20" t="n">
-        <v>48.31</v>
+        <v>48.34</v>
       </c>
       <c r="N20" t="n">
-        <v>17</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
chore(handoff): refresh PLAN.md for the §17/§18 arc + flush pipeline run-state
PLAN.md updated to current state (2026-06-29, 378 tests, @5fa1050): the §17
justified-P/NAV diagnostic + §18 normal-rate layer recorded as DONE; Open threads
rewritten to the P1 follow-ons (§18.5b orderbook, §18.5a Baltic data, product
LR1/Handysize/Handymax marks, the curve.newbuild NAV-layer thread, P3 guards);
the completed Post-Panamax/charter threads removed.

Flushes the decision-log model-state prepends + regenerated per-name outputs from
this arc's verification runs. NO headline FV change (drift gate 0; cycle.py frozen) —
these are non-material run-state refreshes, committed so the tree is clean for handoff.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -1135,7 +1135,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>HAFN</t>
+          <t>SB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1144,23 +1144,23 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.95</v>
+        <v>0.88</v>
       </c>
       <c r="D14" t="n">
-        <v>1.318</v>
+        <v>0.802</v>
       </c>
       <c r="E14" t="n">
-        <v>-15.2</v>
+        <v>46.3</v>
       </c>
       <c r="F14" t="n">
-        <v>-1.9</v>
+        <v>29</v>
       </c>
       <c r="G14" t="n">
-        <v>11.4</v>
+        <v>11.6</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>TRIM/SHORT (overvalued)</t>
+          <t>BUY (undervalued)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>87353</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>29992</v>
+        <v>2688</v>
       </c>
       <c r="L14" t="n">
-        <v>5.91</v>
+        <v>9.35</v>
       </c>
       <c r="M14" t="n">
-        <v>7.76</v>
+        <v>7.13</v>
       </c>
       <c r="N14" t="n">
-        <v>26.6</v>
+        <v>-34.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GNK</t>
+          <t>HAFN</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1196,23 +1196,23 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.87</v>
+        <v>0.95</v>
       </c>
       <c r="D15" t="n">
-        <v>1.08</v>
+        <v>1.318</v>
       </c>
       <c r="E15" t="n">
-        <v>1.9</v>
+        <v>-15.2</v>
       </c>
       <c r="F15" t="n">
-        <v>6.5</v>
+        <v>-1.9</v>
       </c>
       <c r="G15" t="n">
-        <v>11</v>
+        <v>11.4</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>HOLD (fairly valued)</t>
+          <t>TRIM/SHORT (overvalued)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1221,50 +1221,50 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>22647</v>
+        <v>87353</v>
       </c>
       <c r="K15" t="n">
-        <v>12051</v>
+        <v>29992</v>
       </c>
       <c r="L15" t="n">
-        <v>24.02</v>
+        <v>5.91</v>
       </c>
       <c r="M15" t="n">
-        <v>26.16</v>
+        <v>7.76</v>
       </c>
       <c r="N15" t="n">
-        <v>9.1</v>
+        <v>26.6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>INSW</t>
+          <t>GNK</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>WHOLE-COMPANY (hybrid aggregation)</t>
+          <t>whole-company</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.98</v>
+        <v>0.87</v>
       </c>
       <c r="D16" t="n">
-        <v>1.542</v>
+        <v>1.08</v>
       </c>
       <c r="E16" t="n">
-        <v>-22.8</v>
+        <v>1.9</v>
       </c>
       <c r="F16" t="n">
-        <v>-6</v>
+        <v>6.5</v>
       </c>
       <c r="G16" t="n">
-        <v>10.8</v>
+        <v>11</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>TRIM/SHORT (overvalued)</t>
+          <t>HOLD (fairly valued)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1273,50 +1273,50 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>276426</v>
+        <v>22647</v>
       </c>
       <c r="K16" t="n">
-        <v>71380</v>
+        <v>12051</v>
       </c>
       <c r="L16" t="n">
-        <v>61.34</v>
+        <v>24.02</v>
       </c>
       <c r="M16" t="n">
-        <v>88.12</v>
+        <v>26.16</v>
       </c>
       <c r="N16" t="n">
-        <v>33.7</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SB</t>
+          <t>INSW</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>whole-company</t>
+          <t>WHOLE-COMPANY (hybrid aggregation)</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.88</v>
+        <v>0.98</v>
       </c>
       <c r="D17" t="n">
-        <v>0.783</v>
+        <v>1.542</v>
       </c>
       <c r="E17" t="n">
-        <v>49</v>
+        <v>-22.8</v>
       </c>
       <c r="F17" t="n">
-        <v>29.5</v>
+        <v>-6</v>
       </c>
       <c r="G17" t="n">
-        <v>10</v>
+        <v>10.8</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>BUY (undervalued)</t>
+          <t>TRIM/SHORT (overvalued)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1325,19 +1325,19 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>276426</v>
       </c>
       <c r="K17" t="n">
-        <v>11482</v>
+        <v>71380</v>
       </c>
       <c r="L17" t="n">
-        <v>9.52</v>
+        <v>61.34</v>
       </c>
       <c r="M17" t="n">
-        <v>7.03</v>
+        <v>88.12</v>
       </c>
       <c r="N17" t="n">
-        <v>-39</v>
+        <v>33.7</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
chore(refresh): 2026-06-30 daily price refresh + baseline re-ratify (band flips reviewed)
Broad shipping down day (many names -7% to -22%; ASC/STNG flagged >15%, not applied).
All moves ΔNAV 0% — pure price drift. Two position-band flips reviewed and accepted as
trivial price-driven boundary-crossings (annotated in their logs, NOT swept):
  - DHT TRIM/SHORT->HOLD: -4% price, EV -7.7%->-3.9%; a §12 cycle-position read anyway.
  - FLNG HOLD->BUY: -4.2% price, EV +4.7%->+9.3%; GOVERNED-WIDE structural-class, wide band.
Baseline re-ratified at 06-30 prices; drift gate green. Separate from the NAT reconciliation
(committed earlier at the committed price vintage) — market drift kept out of the sourcing commit.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -523,16 +523,16 @@
         <v>0.34</v>
       </c>
       <c r="D2" t="n">
-        <v>1.127</v>
+        <v>1.118</v>
       </c>
       <c r="E2" t="n">
-        <v>83.09999999999999</v>
+        <v>85.2</v>
       </c>
       <c r="F2" t="n">
-        <v>97.8</v>
+        <v>99</v>
       </c>
       <c r="G2" t="n">
-        <v>112.5</v>
+        <v>112.8</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -554,10 +554,10 @@
         <v>65.48999999999999</v>
       </c>
       <c r="M2" t="n">
-        <v>75.98</v>
+        <v>75.25</v>
       </c>
       <c r="N2" t="n">
-        <v>29.3</v>
+        <v>27.6</v>
       </c>
     </row>
     <row r="3">
@@ -627,16 +627,16 @@
         <v>0.67</v>
       </c>
       <c r="D4" t="n">
-        <v>1.125</v>
+        <v>1.117</v>
       </c>
       <c r="E4" t="n">
-        <v>34.8</v>
+        <v>36.4</v>
       </c>
       <c r="F4" t="n">
-        <v>47.8</v>
+        <v>48.7</v>
       </c>
       <c r="G4" t="n">
-        <v>60.8</v>
+        <v>61.1</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>17.16</v>
       </c>
       <c r="M4" t="n">
-        <v>20.47</v>
+        <v>20.26</v>
       </c>
       <c r="N4" t="n">
-        <v>26</v>
+        <v>24.7</v>
       </c>
     </row>
     <row r="5">
@@ -679,16 +679,16 @@
         <v>0.9</v>
       </c>
       <c r="D5" t="n">
-        <v>0.951</v>
+        <v>0.956</v>
       </c>
       <c r="E5" t="n">
-        <v>72</v>
+        <v>68.2</v>
       </c>
       <c r="F5" t="n">
-        <v>61</v>
+        <v>58.6</v>
       </c>
       <c r="G5" t="n">
-        <v>50</v>
+        <v>48.9</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -710,10 +710,10 @@
         <v>35.91</v>
       </c>
       <c r="M5" t="n">
-        <v>31.3</v>
+        <v>31.8</v>
       </c>
       <c r="N5" t="n">
-        <v>-22.1</v>
+        <v>-19.2</v>
       </c>
     </row>
     <row r="6">
@@ -731,16 +731,16 @@
         <v>0.7</v>
       </c>
       <c r="D6" t="n">
-        <v>1.267</v>
+        <v>1.373</v>
       </c>
       <c r="E6" t="n">
-        <v>14.1</v>
+        <v>5.8</v>
       </c>
       <c r="F6" t="n">
-        <v>26.5</v>
+        <v>21.8</v>
       </c>
       <c r="G6" t="n">
-        <v>38.8</v>
+        <v>37.9</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>10829</v>
+        <v>38043</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -762,10 +762,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>97.31999999999999</v>
+        <v>104.22</v>
       </c>
       <c r="N6" t="n">
-        <v>24.7</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -783,16 +783,16 @@
         <v>0.74</v>
       </c>
       <c r="D7" t="n">
-        <v>1.116</v>
+        <v>1.112</v>
       </c>
       <c r="E7" t="n">
-        <v>14.1</v>
+        <v>14.9</v>
       </c>
       <c r="F7" t="n">
-        <v>24.2</v>
+        <v>24.6</v>
       </c>
       <c r="G7" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>41510</v>
+        <v>39378</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -814,16 +814,16 @@
         <v>16.07</v>
       </c>
       <c r="M7" t="n">
-        <v>18.91</v>
+        <v>18.8</v>
       </c>
       <c r="N7" t="n">
-        <v>20.1</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TNK</t>
+          <t>GSL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -832,19 +832,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="D8" t="n">
-        <v>1.203</v>
+        <v>1.237</v>
       </c>
       <c r="E8" t="n">
-        <v>20.6</v>
+        <v>8</v>
       </c>
       <c r="F8" t="n">
-        <v>26.8</v>
+        <v>20</v>
       </c>
       <c r="G8" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -863,19 +863,19 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>79.59</v>
+        <v>40.59</v>
       </c>
       <c r="M8" t="n">
-        <v>87.75</v>
+        <v>49.64</v>
       </c>
       <c r="N8" t="n">
-        <v>12.4</v>
+        <v>24.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GSL</t>
+          <t>TNK</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -884,19 +884,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="D9" t="n">
-        <v>1.241</v>
+        <v>1.341</v>
       </c>
       <c r="E9" t="n">
-        <v>7.6</v>
+        <v>12.4</v>
       </c>
       <c r="F9" t="n">
-        <v>19.7</v>
+        <v>22.1</v>
       </c>
       <c r="G9" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -909,19 +909,19 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>10261</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>40.59</v>
+        <v>79.59</v>
       </c>
       <c r="M9" t="n">
-        <v>49.78</v>
+        <v>93.28</v>
       </c>
       <c r="N9" t="n">
-        <v>24.4</v>
+        <v>19.3</v>
       </c>
     </row>
     <row r="10">
@@ -939,16 +939,16 @@
         <v>0.83</v>
       </c>
       <c r="D10" t="n">
-        <v>1.174</v>
+        <v>1.165</v>
       </c>
       <c r="E10" t="n">
-        <v>3.8</v>
+        <v>4.8</v>
       </c>
       <c r="F10" t="n">
-        <v>14.3</v>
+        <v>14.9</v>
       </c>
       <c r="G10" t="n">
-        <v>24.7</v>
+        <v>24.9</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -961,19 +961,19 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>48537</v>
+        <v>46693</v>
       </c>
       <c r="K10" t="n">
-        <v>7012</v>
+        <v>7144</v>
       </c>
       <c r="L10" t="n">
         <v>27.32</v>
       </c>
       <c r="M10" t="n">
-        <v>32.81</v>
+        <v>32.55</v>
       </c>
       <c r="N10" t="n">
-        <v>20.9</v>
+        <v>20.1</v>
       </c>
     </row>
     <row r="11">
@@ -1043,16 +1043,16 @@
         <v>0.85</v>
       </c>
       <c r="D12" t="n">
-        <v>2.144</v>
+        <v>1.977</v>
       </c>
       <c r="E12" t="n">
-        <v>-51.9</v>
+        <v>-39.9</v>
       </c>
       <c r="F12" t="n">
-        <v>-14.8</v>
+        <v>-9.300000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>22.3</v>
+        <v>21.2</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1065,19 +1065,19 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>397445</v>
+        <v>360646</v>
       </c>
       <c r="K12" t="n">
-        <v>836</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>2.78</v>
+        <v>3.33</v>
       </c>
       <c r="M12" t="n">
-        <v>7.07</v>
+        <v>6.71</v>
       </c>
       <c r="N12" t="n">
-        <v>74.2</v>
+        <v>61.1</v>
       </c>
     </row>
     <row r="13">
@@ -1095,16 +1095,16 @@
         <v>0.82</v>
       </c>
       <c r="D13" t="n">
-        <v>1.019</v>
+        <v>1.03</v>
       </c>
       <c r="E13" t="n">
-        <v>15.1</v>
+        <v>13.6</v>
       </c>
       <c r="F13" t="n">
-        <v>16.4</v>
+        <v>15.5</v>
       </c>
       <c r="G13" t="n">
-        <v>17.6</v>
+        <v>17.5</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1117,19 +1117,19 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>7455</v>
+        <v>8819</v>
       </c>
       <c r="K13" t="n">
-        <v>4797</v>
+        <v>4716</v>
       </c>
       <c r="L13" t="n">
         <v>28.37</v>
       </c>
       <c r="M13" t="n">
-        <v>28.98</v>
+        <v>29.33</v>
       </c>
       <c r="N13" t="n">
-        <v>2.5</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="14">
@@ -1147,16 +1147,16 @@
         <v>0.88</v>
       </c>
       <c r="D14" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.804</v>
       </c>
       <c r="E14" t="n">
-        <v>56.8</v>
+        <v>58</v>
       </c>
       <c r="F14" t="n">
-        <v>34.7</v>
+        <v>35.3</v>
       </c>
       <c r="G14" t="n">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1172,16 +1172,16 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>2502</v>
+        <v>2497</v>
       </c>
       <c r="L14" t="n">
         <v>9.970000000000001</v>
       </c>
       <c r="M14" t="n">
-        <v>7.16</v>
+        <v>7.11</v>
       </c>
       <c r="N14" t="n">
-        <v>-44.2</v>
+        <v>-45.3</v>
       </c>
     </row>
     <row r="15">
@@ -1199,16 +1199,16 @@
         <v>0.95</v>
       </c>
       <c r="D15" t="n">
-        <v>1.301</v>
+        <v>1.266</v>
       </c>
       <c r="E15" t="n">
-        <v>-13.8</v>
+        <v>-11</v>
       </c>
       <c r="F15" t="n">
-        <v>-1.1</v>
+        <v>0.7</v>
       </c>
       <c r="G15" t="n">
-        <v>11.7</v>
+        <v>12.4</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1221,19 +1221,19 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>83976</v>
+        <v>77221</v>
       </c>
       <c r="K15" t="n">
-        <v>29748</v>
+        <v>29262</v>
       </c>
       <c r="L15" t="n">
         <v>5.91</v>
       </c>
       <c r="M15" t="n">
-        <v>7.66</v>
+        <v>7.46</v>
       </c>
       <c r="N15" t="n">
-        <v>25.5</v>
+        <v>23.3</v>
       </c>
     </row>
     <row r="16">
@@ -1251,16 +1251,16 @@
         <v>0.98</v>
       </c>
       <c r="D16" t="n">
-        <v>1.509</v>
+        <v>1.485</v>
       </c>
       <c r="E16" t="n">
-        <v>-21.2</v>
+        <v>-19.9</v>
       </c>
       <c r="F16" t="n">
-        <v>-5</v>
+        <v>-4.2</v>
       </c>
       <c r="G16" t="n">
-        <v>11.2</v>
+        <v>11.4</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1273,19 +1273,19 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>262650</v>
+        <v>252764</v>
       </c>
       <c r="K16" t="n">
-        <v>70065</v>
+        <v>69122</v>
       </c>
       <c r="L16" t="n">
         <v>61.34</v>
       </c>
       <c r="M16" t="n">
-        <v>86.5</v>
+        <v>85.33</v>
       </c>
       <c r="N16" t="n">
-        <v>32.3</v>
+        <v>31.3</v>
       </c>
     </row>
     <row r="17">
@@ -1303,16 +1303,16 @@
         <v>0.87</v>
       </c>
       <c r="D17" t="n">
-        <v>1.109</v>
+        <v>1.124</v>
       </c>
       <c r="E17" t="n">
-        <v>-1.4</v>
+        <v>-2.9</v>
       </c>
       <c r="F17" t="n">
-        <v>4.6</v>
+        <v>3.7</v>
       </c>
       <c r="G17" t="n">
-        <v>10.6</v>
+        <v>10.4</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1325,19 +1325,19 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>26698</v>
+        <v>28690</v>
       </c>
       <c r="K17" t="n">
-        <v>12255</v>
+        <v>12311</v>
       </c>
       <c r="L17" t="n">
         <v>24.05</v>
       </c>
       <c r="M17" t="n">
-        <v>26.97</v>
+        <v>27.36</v>
       </c>
       <c r="N17" t="n">
-        <v>11.9</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="18">
@@ -1355,16 +1355,16 @@
         <v>0.62</v>
       </c>
       <c r="D18" t="n">
-        <v>0.915</v>
+        <v>0.889</v>
       </c>
       <c r="E18" t="n">
-        <v>13.6</v>
+        <v>16.3</v>
       </c>
       <c r="F18" t="n">
-        <v>9.699999999999999</v>
+        <v>11.2</v>
       </c>
       <c r="G18" t="n">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1377,19 +1377,19 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>5949</v>
+        <v>3273</v>
       </c>
       <c r="K18" t="n">
-        <v>14626</v>
+        <v>14550</v>
       </c>
       <c r="L18" t="n">
         <v>20.43</v>
       </c>
       <c r="M18" t="n">
-        <v>19.03</v>
+        <v>18.61</v>
       </c>
       <c r="N18" t="n">
-        <v>-7.8</v>
+        <v>-10.3</v>
       </c>
     </row>
     <row r="19">
@@ -1407,20 +1407,20 @@
         <v>1.09</v>
       </c>
       <c r="D19" t="n">
-        <v>1.113</v>
+        <v>1.074</v>
       </c>
       <c r="E19" t="n">
-        <v>-7.7</v>
+        <v>-3.9</v>
       </c>
       <c r="F19" t="n">
-        <v>-2.9</v>
+        <v>-0.6</v>
       </c>
       <c r="G19" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>TRIM/SHORT (overvalued)</t>
+          <t>HOLD (fairly valued)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1429,19 +1429,19 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>310818</v>
+        <v>260972</v>
       </c>
       <c r="K19" t="n">
-        <v>194121</v>
+        <v>184868</v>
       </c>
       <c r="L19" t="n">
         <v>15.77</v>
       </c>
       <c r="M19" t="n">
-        <v>17.41</v>
+        <v>16.84</v>
       </c>
       <c r="N19" t="n">
-        <v>9.6</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="20">
@@ -1459,16 +1459,16 @@
         <v>1.04</v>
       </c>
       <c r="D20" t="n">
-        <v>1.144</v>
+        <v>1.125</v>
       </c>
       <c r="E20" t="n">
-        <v>-19.6</v>
+        <v>-17.4</v>
       </c>
       <c r="F20" t="n">
-        <v>-12</v>
+        <v>-10.6</v>
       </c>
       <c r="G20" t="n">
-        <v>-4.3</v>
+        <v>-3.8</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1481,19 +1481,19 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>157594</v>
+        <v>140273</v>
       </c>
       <c r="K20" t="n">
-        <v>49535</v>
+        <v>46859</v>
       </c>
       <c r="L20" t="n">
         <v>2.11</v>
       </c>
       <c r="M20" t="n">
-        <v>2.51</v>
+        <v>2.45</v>
       </c>
       <c r="N20" t="n">
-        <v>15.3</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="21">
@@ -1511,16 +1511,16 @@
         <v>1.2</v>
       </c>
       <c r="D21" t="n">
-        <v>1.145</v>
+        <v>1.123</v>
       </c>
       <c r="E21" t="n">
-        <v>-18.7</v>
+        <v>-16.5</v>
       </c>
       <c r="F21" t="n">
-        <v>-11.8</v>
+        <v>-10.4</v>
       </c>
       <c r="G21" t="n">
-        <v>-4.9</v>
+        <v>-4.4</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1533,19 +1533,19 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>338039</v>
+        <v>316083</v>
       </c>
       <c r="K21" t="n">
-        <v>227490</v>
+        <v>221830</v>
       </c>
       <c r="L21" t="n">
         <v>28.82</v>
       </c>
       <c r="M21" t="n">
-        <v>33.72</v>
+        <v>33</v>
       </c>
       <c r="N21" t="n">
-        <v>13.8</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="22">
@@ -1563,16 +1563,16 @@
         <v>1.21</v>
       </c>
       <c r="D22" t="n">
-        <v>1.13</v>
+        <v>1.139</v>
       </c>
       <c r="E22" t="n">
-        <v>-19</v>
+        <v>-19.9</v>
       </c>
       <c r="F22" t="n">
-        <v>-13</v>
+        <v>-13.5</v>
       </c>
       <c r="G22" t="n">
-        <v>-7.1</v>
+        <v>-7.2</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1585,19 +1585,19 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>292039</v>
+        <v>299354</v>
       </c>
       <c r="K22" t="n">
-        <v>211357</v>
+        <v>213281</v>
       </c>
       <c r="L22" t="n">
         <v>40.17</v>
       </c>
       <c r="M22" t="n">
-        <v>46.09</v>
+        <v>46.49</v>
       </c>
       <c r="N22" t="n">
-        <v>11.9</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="23">
@@ -1615,20 +1615,20 @@
         <v>1.37</v>
       </c>
       <c r="D23" t="n">
-        <v>0.869</v>
+        <v>0.852</v>
       </c>
       <c r="E23" t="n">
-        <v>4.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F23" t="n">
-        <v>-6.5</v>
+        <v>-3.9</v>
       </c>
       <c r="G23" t="n">
-        <v>-17.7</v>
+        <v>-17.1</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>HOLD (fairly valued)</t>
+          <t>BUY (undervalued)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1637,19 +1637,19 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>124006</v>
+        <v>57631</v>
       </c>
       <c r="K23" t="n">
-        <v>453302</v>
+        <v>428722</v>
       </c>
       <c r="L23" t="n">
         <v>30.67</v>
       </c>
       <c r="M23" t="n">
-        <v>24.11</v>
+        <v>23.28</v>
       </c>
       <c r="N23" t="n">
-        <v>-22.4</v>
+        <v>-26.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(p1c): MR secondhand line RESUMED — age-0 54→55.0 on the 2026-07-13 xclusiv MR2 Resale, basis → resale-uniform; thread (d) + P1c state into PLAN/CHANGELOG
crude-tanker-fv. Wiring per the frozen prereg (mr_secondhand_resumption_2026-07-15.md):
xclusiv extract +MR row (per-row 07-13 vintage, annotated), curve/prompt_resale 55.0M,
basis_status resale-uniform, XCLUSIV_WIRED += MR, AGE0_BASIS exception retired (deliberate
loud flip). Landed exactly on the pre-registered band: TEN sole mover +$1.94M (+0.07%,
88.70→88.76), zero flips/tier/basis-composite changes, drift gate 25/0 UNEXPLAINED, suite
588+16x, no re-ratify. Consequence recorded: LR1 = TRMD's and INSW's LAST basis blocker
(fork staged). Includes the expected pipeline model-state churn (25 logs) + outputs regen.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -523,13 +523,13 @@
         <v>0.34</v>
       </c>
       <c r="D2" t="n">
-        <v>1.218</v>
+        <v>1.217</v>
       </c>
       <c r="E2" t="n">
-        <v>44.9</v>
+        <v>45</v>
       </c>
       <c r="F2" t="n">
-        <v>65.40000000000001</v>
+        <v>65.5</v>
       </c>
       <c r="G2" t="n">
         <v>86</v>
@@ -551,13 +551,13 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>57.6</v>
+        <v>57.64</v>
       </c>
       <c r="M2" t="n">
         <v>73.93000000000001</v>
       </c>
       <c r="N2" t="n">
-        <v>41.1</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
chore(logs): pipeline auto-entries from the reconciliation verification runs
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -523,16 +523,16 @@
         <v>0.34</v>
       </c>
       <c r="D2" t="n">
-        <v>1.217</v>
+        <v>1.24</v>
       </c>
       <c r="E2" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F2" t="n">
-        <v>65.5</v>
+        <v>63.6</v>
       </c>
       <c r="G2" t="n">
-        <v>86</v>
+        <v>85.2</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -551,13 +551,13 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>57.64</v>
+        <v>56.46</v>
       </c>
       <c r="M2" t="n">
-        <v>73.93000000000001</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>41</v>
+        <v>43.1</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
feat(ppmx): §9.9 fit SEEDED (owner: 'seed the PPMX §9.9 fit') — 5-print sample wired, anchors 34/26 -> 33.56/24.33, SB -1.5% NAV in-band; MARK_WIDE both nodes + ppmx_txn_refit armed
crude-tanker-fv. Per the frozen prereg: transactions/post_panamax.yaml (5 prints, one
tc_attached); MARK_WIDE_NODES Post-Panamax (LOO 10yr 18.1-30.6, 5yr 21.1-43.7 — the
15-16 age cluster); refit trigger armed (>=8 prints incl >=2 at age <=12); CLAUDE.md
known-limit line retired-to-seeded; sb_log checkpoint entry (the holding card's
pre-registered PPMX falsifier checkpoint: error REAL but SMALL, falsifier NOT fired,
BUY stands); old-age overhang residual (~+28% at ages 15-16) registered as the refit's
methodology fork. Gate: SB -1.5%/-1.8pp sub-bar stable, 0 UNEXPLAINED, sole mover.
Family sidecar re-run at the new basis. SB tier boundary call (flag-not-cap
recommended, 25.8% fleet-value share) = owner cell at the next ratify.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -1095,13 +1095,13 @@
         <v>0.88</v>
       </c>
       <c r="D13" t="n">
-        <v>0.854</v>
+        <v>0.861</v>
       </c>
       <c r="E13" t="n">
-        <v>40.8</v>
+        <v>38.9</v>
       </c>
       <c r="F13" t="n">
-        <v>25.5</v>
+        <v>24.6</v>
       </c>
       <c r="G13" t="n">
         <v>10.3</v>
@@ -1120,16 +1120,16 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>992</v>
+        <v>978</v>
       </c>
       <c r="L13" t="n">
-        <v>9.6</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="M13" t="n">
         <v>7.52</v>
       </c>
       <c r="N13" t="n">
-        <v>-30.5</v>
+        <v>-28.6</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
refresh(SB): recompute — NAV $10.07->$10.73 (+6.6%), BAND MISS by 0.6% -> HALTED+INVESTIGATED per prereg: inputs verify clean; attribution = deliveries + 4 new orders valued at the Pana age-0 anchor ($46.0M) which live young-Pana evidence (Nord 37.5 @4y, MB ladder NB 37.0) prices 15-20% lower — curve NOT tuned, question routed to the ladder-ingest/young-end review; honesty line in sb_log. BUY stands EV +29.4%. Pins: fleet 21/16/7 + 9NB, scrubber ledgers 20->19 both copies (Xenia HFS), refresh test census-dynamic
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -1095,16 +1095,16 @@
         <v>0.88</v>
       </c>
       <c r="D13" t="n">
-        <v>0.927</v>
+        <v>0.891</v>
       </c>
       <c r="E13" t="n">
-        <v>21.3</v>
+        <v>29.4</v>
       </c>
       <c r="F13" t="n">
-        <v>14.7</v>
+        <v>19.1</v>
       </c>
       <c r="G13" t="n">
-        <v>8.199999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1120,16 +1120,16 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>529</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>9.470000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="M13" t="n">
-        <v>8.449999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="N13" t="n">
-        <v>-13.1</v>
+        <v>-20.4</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
refresh(TNK): recompute — NAV $77.73->$81.48 (+4.8%) INSIDE the ±8% band; point estimate high ~3.7% (the VLCC's curve mark ~$88M sits ~4% ABOVE its realized $84.5M — a rare issuer-REALIZED old-age corroboration, routed to the curve review not tuned) and the no-flip prediction was WRONG (TRIM/SHORT->HOLD, FV-led, band-mech). TIER VALIDATED-TIGHT->GOVERNED-WIDE·read-flips: at fair value the §9.10 family straddles the boundary — registered in provenance + PLAN. TNK newbuild specs registered (eco §3.1 rule, scrubber FALSE — no filing statement, peer-trap rule). test_verdict_prose de-hardwired (it asserted 'nothing hardwired' via a literal TNK list)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -823,7 +823,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ASC</t>
+          <t>TNK</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -832,19 +832,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="D8" t="n">
-        <v>1.349</v>
+        <v>1.562</v>
       </c>
       <c r="E8" t="n">
-        <v>-3.2</v>
+        <v>-3.8</v>
       </c>
       <c r="F8" t="n">
-        <v>10.4</v>
+        <v>10.2</v>
       </c>
       <c r="G8" t="n">
-        <v>24</v>
+        <v>24.1</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -857,25 +857,25 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>30382</v>
+        <v>54688</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>16.85</v>
+        <v>76.95</v>
       </c>
       <c r="M8" t="n">
-        <v>21.57</v>
+        <v>99.23999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>27.1</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TNK</t>
+          <t>ASC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -884,23 +884,23 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="D9" t="n">
-        <v>1.689</v>
+        <v>1.349</v>
       </c>
       <c r="E9" t="n">
-        <v>-7.8</v>
+        <v>-3.2</v>
       </c>
       <c r="F9" t="n">
-        <v>7.8</v>
+        <v>10.4</v>
       </c>
       <c r="G9" t="n">
-        <v>23.5</v>
+        <v>24</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>TRIM/SHORT (overvalued)</t>
+          <t>HOLD (fairly valued)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -909,19 +909,19 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>87258</v>
+        <v>30382</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>73.69</v>
+        <v>16.85</v>
       </c>
       <c r="M9" t="n">
-        <v>98.75</v>
+        <v>21.57</v>
       </c>
       <c r="N9" t="n">
-        <v>31.3</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
REVERT+RECORD: the three 2026-07-31 Q2 refreshes were HALF-APPLIED — balance sheets are quarter-keyed (exact path, no fallback) but fleet manifests are not, so on a 2026-Q1 run the asset side went live and the liability side was never read (ASC: 4 NB hulls on-curve vs commitments still 0 -> +16.9% artifact vs ~-2.9% paired). Manifests + their pins REVERTED to coherent Q1 state (SB 10.07 / TNK 77.73 / ASC 17.82 restored); the Q2 balance sheets + newbuild_specs KEPT and STAGED for a planned cluster transition. VOID banners on the three logs (attributions demoted to hypotheses), design gap + two candidate fixes recorded, CLAUDE.md snapshot-integrity rule extended to APPLICATION, coherence guard task spawned
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -823,7 +823,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TNK</t>
+          <t>ASC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -832,19 +832,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="D8" t="n">
-        <v>1.562</v>
+        <v>1.349</v>
       </c>
       <c r="E8" t="n">
-        <v>-3.8</v>
+        <v>-3.2</v>
       </c>
       <c r="F8" t="n">
-        <v>10.2</v>
+        <v>10.4</v>
       </c>
       <c r="G8" t="n">
-        <v>24.1</v>
+        <v>24</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -857,25 +857,25 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>54688</v>
+        <v>30382</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>76.95</v>
+        <v>16.85</v>
       </c>
       <c r="M8" t="n">
-        <v>99.23999999999999</v>
+        <v>21.57</v>
       </c>
       <c r="N8" t="n">
-        <v>27.9</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ASC</t>
+          <t>TNK</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -884,23 +884,23 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="D9" t="n">
-        <v>1.349</v>
+        <v>1.689</v>
       </c>
       <c r="E9" t="n">
-        <v>-3.2</v>
+        <v>-7.8</v>
       </c>
       <c r="F9" t="n">
-        <v>10.4</v>
+        <v>7.8</v>
       </c>
       <c r="G9" t="n">
-        <v>24</v>
+        <v>23.5</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>HOLD (fairly valued)</t>
+          <t>TRIM/SHORT (overvalued)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -909,19 +909,19 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>30382</v>
+        <v>87258</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>16.85</v>
+        <v>73.69</v>
       </c>
       <c r="M9" t="n">
-        <v>21.57</v>
+        <v>98.75</v>
       </c>
       <c r="N9" t="n">
-        <v>27.1</v>
+        <v>31.3</v>
       </c>
     </row>
     <row r="10">
@@ -1095,16 +1095,16 @@
         <v>0.88</v>
       </c>
       <c r="D13" t="n">
-        <v>0.891</v>
+        <v>0.927</v>
       </c>
       <c r="E13" t="n">
-        <v>29.4</v>
+        <v>21.3</v>
       </c>
       <c r="F13" t="n">
-        <v>19.1</v>
+        <v>14.7</v>
       </c>
       <c r="G13" t="n">
-        <v>8.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1120,16 +1120,16 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>529</v>
       </c>
       <c r="L13" t="n">
-        <v>10.1</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>8.51</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="N13" t="n">
-        <v>-20.4</v>
+        <v>-13.1</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
chore(outputs): clean-stamp regen after the ECO refresh (at ada1f21)
ECO NAV 37.65 on the committed Q2 surface (4 names at Q2 vintage, 21 lagging,
disclosed); crude family sidecar current at the new point (ECO WEIGHT-ROBUST
TRIM across the family); gate: ECO explained (log-annotated, batch ratify at
end of drain). Suite 633 green + 15 xfailed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -1707,7 +1707,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FRO</t>
+          <t>ECO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1716,19 +1716,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.37</v>
+        <v>1.35</v>
       </c>
       <c r="D25" t="n">
-        <v>1.134</v>
+        <v>1.169</v>
       </c>
       <c r="E25" t="n">
-        <v>-41.8</v>
+        <v>-42.3</v>
       </c>
       <c r="F25" t="n">
-        <v>-36.8</v>
+        <v>-36.9</v>
       </c>
       <c r="G25" t="n">
-        <v>-31.8</v>
+        <v>-31.6</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1741,25 +1741,25 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>440847</v>
+        <v>421886</v>
       </c>
       <c r="K25" t="n">
-        <v>339112</v>
+        <v>319860</v>
       </c>
       <c r="L25" t="n">
-        <v>23.15</v>
+        <v>35.69</v>
       </c>
       <c r="M25" t="n">
-        <v>27.11</v>
+        <v>42.32</v>
       </c>
       <c r="N25" t="n">
-        <v>10</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ECO</t>
+          <t>FRO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1768,19 +1768,19 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1.35</v>
+        <v>1.37</v>
       </c>
       <c r="D26" t="n">
-        <v>1.232</v>
+        <v>1.134</v>
       </c>
       <c r="E26" t="n">
-        <v>-47.4</v>
+        <v>-41.8</v>
       </c>
       <c r="F26" t="n">
-        <v>-39.9</v>
+        <v>-36.8</v>
       </c>
       <c r="G26" t="n">
-        <v>-32.4</v>
+        <v>-31.8</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1793,19 +1793,19 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>466032</v>
+        <v>440847</v>
       </c>
       <c r="K26" t="n">
-        <v>323230</v>
+        <v>339112</v>
       </c>
       <c r="L26" t="n">
-        <v>32.57</v>
+        <v>23.15</v>
       </c>
       <c r="M26" t="n">
-        <v>41.81</v>
+        <v>27.11</v>
       </c>
       <c r="N26" t="n">
-        <v>14.9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(outputs): clean-stamp regen after the CCEC refresh (at 2322242)
CCEC NAV 25.70 / EV +50.7% BUY on the committed Q2 surface (5 names at Q2
vintage, 20 lagging, disclosed); LNG family sidecar current. Gate 0/0 on the
ECO+CCEC-ratified baseline. Suite 633 green + 15 xfailed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -575,16 +575,16 @@
         <v>0.9</v>
       </c>
       <c r="D3" t="n">
-        <v>0.967</v>
+        <v>0.991</v>
       </c>
       <c r="E3" t="n">
-        <v>60.5</v>
+        <v>50.7</v>
       </c>
       <c r="F3" t="n">
-        <v>53.7</v>
+        <v>48.9</v>
       </c>
       <c r="G3" t="n">
-        <v>46.9</v>
+        <v>47.1</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -603,13 +603,13 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>35.91</v>
+        <v>33.7</v>
       </c>
       <c r="M3" t="n">
-        <v>32.86</v>
+        <v>32.91</v>
       </c>
       <c r="N3" t="n">
-        <v>-13.6</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
chore(outputs): clean-stamp regen after the STNG refresh (at 688fb16)
STNG NAV 76.42 / HOLD on the committed Q2 surface (6 names at Q2 vintage,
19 lagging, disclosed); product family sidecar current. Gate 0/0. Suite 634
green + 14 xfailed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -627,16 +627,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>1.474</v>
+        <v>1.552</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>-3.1</v>
       </c>
       <c r="F4" t="n">
-        <v>20.1</v>
+        <v>16.4</v>
       </c>
       <c r="G4" t="n">
-        <v>39.2</v>
+        <v>35.9</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -649,19 +649,19 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>57165</v>
+        <v>71456</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>76.87</v>
+        <v>73.73</v>
       </c>
       <c r="M4" t="n">
-        <v>105.9</v>
+        <v>103.41</v>
       </c>
       <c r="N4" t="n">
-        <v>38.2</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
chore(outputs): clean-stamp regen after the LPG refresh (at a6d40e8)
LPG NAV 35.69 / TRIM/SHORT (rich · cycle) on the committed Q2 surface
(7 names at Q2 vintage, 18 lagging, disclosed); LPG family sidecar current.
Gate 0/0. Suite 634 green + 14 xfailed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -1135,7 +1135,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LPG</t>
+          <t>CMDB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1144,23 +1144,23 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.84</v>
+        <v>0.62</v>
       </c>
       <c r="D14" t="n">
-        <v>1.499</v>
+        <v>0.862</v>
       </c>
       <c r="E14" t="n">
-        <v>-33.2</v>
+        <v>16.8</v>
       </c>
       <c r="F14" t="n">
-        <v>-14.7</v>
+        <v>10.3</v>
       </c>
       <c r="G14" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>TRIM/SHORT (overvalued)</t>
+          <t>BUY (undervalued)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>206288</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>14830</v>
       </c>
       <c r="L14" t="n">
-        <v>30.55</v>
+        <v>20.79</v>
       </c>
       <c r="M14" t="n">
-        <v>47.48</v>
+        <v>18.47</v>
       </c>
       <c r="N14" t="n">
-        <v>37</v>
+        <v>-13</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CMDB</t>
+          <t>LPG</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1196,23 +1196,23 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.62</v>
+        <v>0.84</v>
       </c>
       <c r="D15" t="n">
-        <v>0.862</v>
+        <v>1.569</v>
       </c>
       <c r="E15" t="n">
-        <v>16.8</v>
+        <v>-30.5</v>
       </c>
       <c r="F15" t="n">
-        <v>10.3</v>
+        <v>-13.4</v>
       </c>
       <c r="G15" t="n">
         <v>3.7</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>BUY (undervalued)</t>
+          <t>TRIM/SHORT (overvalued)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1221,19 +1221,19 @@
         </is>
       </c>
       <c r="J15" t="n">
+        <v>223619</v>
+      </c>
+      <c r="K15" t="n">
         <v>0</v>
       </c>
-      <c r="K15" t="n">
-        <v>14830</v>
-      </c>
       <c r="L15" t="n">
-        <v>20.79</v>
+        <v>31.82</v>
       </c>
       <c r="M15" t="n">
-        <v>18.47</v>
+        <v>47.43</v>
       </c>
       <c r="N15" t="n">
-        <v>-13</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(outputs): clean-stamp regen after the GSL refresh (at 2801bb7)
GSL NAV 41.20 / HOLD on the committed Q2 surface (8 names at Q2 vintage, 17
lagging, disclosed). Gate 0/0. Suite 634 green + 15 xfailed (the GSL
convention xfail joins the queue).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -667,7 +667,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ASC</t>
+          <t>GSL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -679,16 +679,16 @@
         <v>0.75</v>
       </c>
       <c r="D5" t="n">
-        <v>1.266</v>
+        <v>1.324</v>
       </c>
       <c r="E5" t="n">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
       <c r="F5" t="n">
-        <v>15.6</v>
+        <v>15.5</v>
       </c>
       <c r="G5" t="n">
-        <v>28.7</v>
+        <v>29.7</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -701,25 +701,25 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>21597</v>
+        <v>16874</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>17.11</v>
+        <v>43.02</v>
       </c>
       <c r="M5" t="n">
-        <v>21.51</v>
+        <v>55.05</v>
       </c>
       <c r="N5" t="n">
-        <v>26.3</v>
+        <v>28.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GSL</t>
+          <t>ASC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -731,13 +731,13 @@
         <v>0.75</v>
       </c>
       <c r="D6" t="n">
-        <v>1.37</v>
+        <v>1.266</v>
       </c>
       <c r="E6" t="n">
-        <v>-4.5</v>
+        <v>2.4</v>
       </c>
       <c r="F6" t="n">
-        <v>12.1</v>
+        <v>15.6</v>
       </c>
       <c r="G6" t="n">
         <v>28.7</v>
@@ -753,19 +753,19 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>75049</v>
+        <v>21597</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>40.54</v>
+        <v>17.11</v>
       </c>
       <c r="M6" t="n">
-        <v>54.62</v>
+        <v>21.51</v>
       </c>
       <c r="N6" t="n">
-        <v>33.2</v>
+        <v>26.3</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
chore(outputs+tests): clean-stamp regen after the DHT refresh (at c9faa9a) + the DHT-specimen test sweep
DHT NAV 13.83 / TRIM/SHORT rich·cycle on the committed Q2 surface (9 names at
Q2 vintage, 16 lagging, disclosed). DHT is the suite's canonical specimen —
34 hardcoded "2026-Q1" load sites across 11 test files swept to BOOK_QUARTER
when its manifest advanced (the pair guard fired at collection, as designed);
value pins re-based with dated comments (fleet_value 2911.35->2842.80 = the
+0.5y age-basis effect; report FV 14.68->14.91); the two coherence tests that
assumed DHT-is-Q1-only now pin their world via _drop_sheets_after / FRO as
the lagging specimen. Gate 0/0 (sub-threshold, unratified by design). Suite
634 green + 15 xfailed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -1615,16 +1615,16 @@
         <v>1.14</v>
       </c>
       <c r="D23" t="n">
-        <v>1.184</v>
+        <v>1.174</v>
       </c>
       <c r="E23" t="n">
-        <v>-29.4</v>
+        <v>-28</v>
       </c>
       <c r="F23" t="n">
-        <v>-23.3</v>
+        <v>-22.4</v>
       </c>
       <c r="G23" t="n">
-        <v>-17.1</v>
+        <v>-16.7</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1637,19 +1637,19 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>453752</v>
+        <v>437369</v>
       </c>
       <c r="K23" t="n">
-        <v>267029</v>
+        <v>266381</v>
       </c>
       <c r="L23" t="n">
-        <v>13.24</v>
+        <v>13.51</v>
       </c>
       <c r="M23" t="n">
-        <v>15.55</v>
+        <v>15.62</v>
       </c>
       <c r="N23" t="n">
-        <v>12.3</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
chore(outputs): clean-stamp regen after the GNK refresh (at HEAD^)
GNK NAV 25.26 / TRIM/SHORT (band-mech flip, rich·cycle relabel downstream) on
the committed Q2 surface (10 names at Q2 vintage, 15 lagging, disclosed);
dry-bulk family sidecar current (GNK WEIGHT-DRIVEN across sets — the
boundary-sitter signature). Gate 0/0. Suite green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -1251,41 +1251,41 @@
         <v>0.89</v>
       </c>
       <c r="D16" t="n">
-        <v>1.078</v>
+        <v>1.1</v>
       </c>
       <c r="E16" t="n">
-        <v>-4.9</v>
+        <v>-7.5</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.8</v>
+        <v>-2.2</v>
       </c>
       <c r="G16" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
+          <t>TRIM/SHORT (overvalued)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
           <t>HOLD (fairly valued)</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>HOLD (fairly valued)</t>
-        </is>
-      </c>
       <c r="J16" t="n">
-        <v>27848</v>
+        <v>32091</v>
       </c>
       <c r="K16" t="n">
-        <v>14242</v>
+        <v>14737</v>
       </c>
       <c r="L16" t="n">
-        <v>24.08</v>
+        <v>23.42</v>
       </c>
       <c r="M16" t="n">
-        <v>26.15</v>
+        <v>26.1</v>
       </c>
       <c r="N16" t="n">
-        <v>8.199999999999999</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
chore(outputs): clean-stamp regen after the SBLK refresh (at HEAD^)
SBLK NAV 32.39 / HOLD (EV +4.6%, 0.4pp under the BUY edge) on the committed
Q2 surface (12 names at Q2 vintage, 13 lagging, disclosed); dry-bulk family
current (SBLK WEIGHT-DRIVEN near the boundary). Gate 0/0. Suite green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -991,16 +991,16 @@
         <v>0.78</v>
       </c>
       <c r="D11" t="n">
-        <v>1.169</v>
+        <v>1.122</v>
       </c>
       <c r="E11" t="n">
-        <v>-1</v>
+        <v>4.6</v>
       </c>
       <c r="F11" t="n">
-        <v>8.4</v>
+        <v>11.3</v>
       </c>
       <c r="G11" t="n">
-        <v>17.8</v>
+        <v>18.1</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1013,19 +1013,19 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>19951</v>
+        <v>13931</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>28.62</v>
+        <v>30.22</v>
       </c>
       <c r="M11" t="n">
-        <v>34.04</v>
+        <v>34.14</v>
       </c>
       <c r="N11" t="n">
-        <v>18.7</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
chore(outputs): clean-stamp regen after the CMDB refresh (at HEAD^) — the Q2 drain surface
13 names at Q2 vintage, 12 lagging (disclosed): the drainable backlog is
COMPLETE. CMDB NAV 31.92 / BUY. Gate 0/0. Suite green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -1135,7 +1135,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CMDB</t>
+          <t>LPG</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1144,23 +1144,23 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.62</v>
+        <v>0.84</v>
       </c>
       <c r="D14" t="n">
-        <v>0.862</v>
+        <v>1.569</v>
       </c>
       <c r="E14" t="n">
-        <v>16.8</v>
+        <v>-30.5</v>
       </c>
       <c r="F14" t="n">
-        <v>10.3</v>
+        <v>-13.4</v>
       </c>
       <c r="G14" t="n">
         <v>3.7</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>BUY (undervalued)</t>
+          <t>TRIM/SHORT (overvalued)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="J14" t="n">
+        <v>223619</v>
+      </c>
+      <c r="K14" t="n">
         <v>0</v>
       </c>
-      <c r="K14" t="n">
-        <v>14830</v>
-      </c>
       <c r="L14" t="n">
-        <v>20.79</v>
+        <v>31.82</v>
       </c>
       <c r="M14" t="n">
-        <v>18.47</v>
+        <v>47.43</v>
       </c>
       <c r="N14" t="n">
-        <v>-13</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LPG</t>
+          <t>CMDB</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1196,23 +1196,23 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.84</v>
+        <v>0.62</v>
       </c>
       <c r="D15" t="n">
-        <v>1.569</v>
+        <v>0.886</v>
       </c>
       <c r="E15" t="n">
-        <v>-30.5</v>
+        <v>14.2</v>
       </c>
       <c r="F15" t="n">
-        <v>-13.4</v>
+        <v>8.9</v>
       </c>
       <c r="G15" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>TRIM/SHORT (overvalued)</t>
+          <t>BUY (undervalued)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1221,19 +1221,19 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>223619</v>
+        <v>2798</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>14918</v>
       </c>
       <c r="L15" t="n">
-        <v>31.82</v>
+        <v>20.33</v>
       </c>
       <c r="M15" t="n">
-        <v>47.43</v>
+        <v>18.44</v>
       </c>
       <c r="N15" t="n">
-        <v>34.1</v>
+        <v>-10.6</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
BRUT absorb regen: first 4-hull run — NAV $4.92, EV +3.6% HOLD, k 0.99 (tightest ever); guards released, forward invariance held; log annotated, NAV pin re-based to the print
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -719,7 +719,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BRUT</t>
+          <t>GSL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -728,50 +728,50 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.86</v>
+        <v>0.75</v>
       </c>
       <c r="D6" t="n">
-        <v>0.871</v>
+        <v>1.382</v>
       </c>
       <c r="E6" t="n">
-        <v>108</v>
+        <v>-3.7</v>
       </c>
       <c r="F6" t="n">
-        <v>70.59999999999999</v>
+        <v>12.2</v>
       </c>
       <c r="G6" t="n">
-        <v>33.3</v>
+        <v>28.1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>HOLD (fairly valued)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>BUY (undervalued)</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>BUY (undervalued)</t>
-        </is>
-      </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>106820</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>10.28</v>
+        <v>42.88</v>
       </c>
       <c r="M6" t="n">
-        <v>6.59</v>
+        <v>57.02</v>
       </c>
       <c r="N6" t="n">
-        <v>-74.7</v>
+        <v>31.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GSL</t>
+          <t>TRMD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -780,23 +780,23 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.75</v>
+        <v>0.86</v>
       </c>
       <c r="D7" t="n">
-        <v>1.382</v>
+        <v>1.148</v>
       </c>
       <c r="E7" t="n">
-        <v>-3.7</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>12.2</v>
+        <v>17.7</v>
       </c>
       <c r="G7" t="n">
-        <v>28.1</v>
+        <v>25.8</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>HOLD (fairly valued)</t>
+          <t>BUY (undervalued)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -805,25 +805,25 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>106820</v>
+        <v>43444</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>9917</v>
       </c>
       <c r="L7" t="n">
-        <v>42.88</v>
+        <v>35.79</v>
       </c>
       <c r="M7" t="n">
-        <v>57.02</v>
+        <v>41.02</v>
       </c>
       <c r="N7" t="n">
-        <v>31.8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TRMD</t>
+          <t>ASC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -832,50 +832,50 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.86</v>
+        <v>0.75</v>
       </c>
       <c r="D8" t="n">
-        <v>1.148</v>
+        <v>1.313</v>
       </c>
       <c r="E8" t="n">
-        <v>9.699999999999999</v>
+        <v>-5.7</v>
       </c>
       <c r="F8" t="n">
-        <v>17.7</v>
+        <v>8.6</v>
       </c>
       <c r="G8" t="n">
-        <v>25.8</v>
+        <v>22.8</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t>TRIM/SHORT (overvalued)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
           <t>BUY (undervalued)</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>BUY (undervalued)</t>
-        </is>
-      </c>
       <c r="J8" t="n">
-        <v>43444</v>
+        <v>28607</v>
       </c>
       <c r="K8" t="n">
-        <v>9917</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>35.79</v>
+        <v>16.38</v>
       </c>
       <c r="M8" t="n">
-        <v>41.02</v>
+        <v>21.31</v>
       </c>
       <c r="N8" t="n">
-        <v>16</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ASC</t>
+          <t>TNK</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -884,19 +884,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="D9" t="n">
-        <v>1.313</v>
+        <v>1.527</v>
       </c>
       <c r="E9" t="n">
-        <v>-5.7</v>
+        <v>-5.4</v>
       </c>
       <c r="F9" t="n">
-        <v>8.6</v>
+        <v>7.6</v>
       </c>
       <c r="G9" t="n">
-        <v>22.8</v>
+        <v>20.6</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>28607</v>
+        <v>130174</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>16.38</v>
+        <v>83.93000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>21.31</v>
+        <v>106.94</v>
       </c>
       <c r="N9" t="n">
-        <v>28.4</v>
+        <v>25.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TNK</t>
+          <t>HAFN</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -936,19 +936,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.8</v>
+        <v>0.92</v>
       </c>
       <c r="D10" t="n">
-        <v>1.527</v>
+        <v>1.553</v>
       </c>
       <c r="E10" t="n">
-        <v>-5.4</v>
+        <v>-22.6</v>
       </c>
       <c r="F10" t="n">
-        <v>7.6</v>
+        <v>-2.7</v>
       </c>
       <c r="G10" t="n">
-        <v>20.6</v>
+        <v>17.2</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -961,25 +961,25 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>130174</v>
+        <v>126841</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>25310</v>
       </c>
       <c r="L10" t="n">
-        <v>83.93000000000001</v>
+        <v>6.56</v>
       </c>
       <c r="M10" t="n">
-        <v>106.94</v>
+        <v>9.92</v>
       </c>
       <c r="N10" t="n">
-        <v>25.9</v>
+        <v>39.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HAFN</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -988,19 +988,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="D11" t="n">
-        <v>1.553</v>
+        <v>2.325</v>
       </c>
       <c r="E11" t="n">
-        <v>-22.6</v>
+        <v>-54.7</v>
       </c>
       <c r="F11" t="n">
-        <v>-2.7</v>
+        <v>-21.6</v>
       </c>
       <c r="G11" t="n">
-        <v>17.2</v>
+        <v>11.4</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1013,25 +1013,25 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>126841</v>
+        <v>667460</v>
       </c>
       <c r="K11" t="n">
-        <v>25310</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>6.56</v>
+        <v>3.07</v>
       </c>
       <c r="M11" t="n">
-        <v>9.92</v>
+        <v>7.54</v>
       </c>
       <c r="N11" t="n">
-        <v>39.8</v>
+        <v>66.09999999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>2343</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1040,23 +1040,23 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.85</v>
+        <v>0.91</v>
       </c>
       <c r="D12" t="n">
-        <v>2.325</v>
+        <v>1.049</v>
       </c>
       <c r="E12" t="n">
-        <v>-54.7</v>
+        <v>1.4</v>
       </c>
       <c r="F12" t="n">
-        <v>-21.6</v>
+        <v>3.8</v>
       </c>
       <c r="G12" t="n">
-        <v>11.4</v>
+        <v>6.2</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>TRIM/SHORT (overvalued)</t>
+          <t>HOLD (fairly valued)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1065,25 +1065,25 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>667460</v>
+        <v>14262</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>11346</v>
       </c>
       <c r="L12" t="n">
-        <v>3.07</v>
+        <v>0.4</v>
       </c>
       <c r="M12" t="n">
-        <v>7.54</v>
+        <v>0.41</v>
       </c>
       <c r="N12" t="n">
-        <v>66.09999999999999</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2343</t>
+          <t>SB</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1092,23 +1092,23 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="D13" t="n">
-        <v>1.049</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="E13" t="n">
-        <v>1.4</v>
+        <v>49.2</v>
       </c>
       <c r="F13" t="n">
-        <v>3.8</v>
+        <v>27.4</v>
       </c>
       <c r="G13" t="n">
-        <v>6.2</v>
+        <v>5.7</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>HOLD (fairly valued)</t>
+          <t>BUY (undervalued)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1117,129 +1117,129 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>14262</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>11346</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0.4</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="M13" t="n">
-        <v>0.41</v>
+        <v>6.75</v>
       </c>
       <c r="N13" t="n">
-        <v>4.8</v>
+        <v>-43.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SB</t>
+          <t>CMBT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>whole-company</t>
+          <t>WHOLE-COMPANY (hybrid aggregation)</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="D14" t="n">
-        <v>0.8120000000000001</v>
+        <v>1.185</v>
       </c>
       <c r="E14" t="n">
-        <v>49.2</v>
+        <v>-21.5</v>
       </c>
       <c r="F14" t="n">
-        <v>27.4</v>
+        <v>-9.9</v>
       </c>
       <c r="G14" t="n">
-        <v>5.7</v>
+        <v>1.7</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
+          <t>TRIM/SHORT (overvalued)</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
           <t>BUY (undervalued)</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>BUY (undervalued)</t>
-        </is>
-      </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>170829</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>28253</v>
       </c>
       <c r="L14" t="n">
-        <v>9.529999999999999</v>
+        <v>14.41</v>
       </c>
       <c r="M14" t="n">
-        <v>6.75</v>
+        <v>18.67</v>
       </c>
       <c r="N14" t="n">
-        <v>-43.5</v>
+        <v>23.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CMBT</t>
+          <t>SBLK</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>WHOLE-COMPANY (hybrid aggregation)</t>
+          <t>whole-company</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.85</v>
+        <v>0.89</v>
       </c>
       <c r="D15" t="n">
-        <v>1.185</v>
+        <v>1.038</v>
       </c>
       <c r="E15" t="n">
-        <v>-21.5</v>
+        <v>-2.3</v>
       </c>
       <c r="F15" t="n">
-        <v>-9.9</v>
+        <v>-0.3</v>
       </c>
       <c r="G15" t="n">
         <v>1.7</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>TRIM/SHORT (overvalued)</t>
+          <t>HOLD (fairly valued)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>BUY (undervalued)</t>
+          <t>HOLD (fairly valued)</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>170829</v>
+        <v>18174</v>
       </c>
       <c r="K15" t="n">
-        <v>28253</v>
+        <v>13478</v>
       </c>
       <c r="L15" t="n">
-        <v>14.41</v>
+        <v>29.79</v>
       </c>
       <c r="M15" t="n">
-        <v>18.67</v>
+        <v>30.99</v>
       </c>
       <c r="N15" t="n">
-        <v>23.2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SBLK</t>
+          <t>BRUT</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1248,19 +1248,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.89</v>
+        <v>1.03</v>
       </c>
       <c r="D16" t="n">
-        <v>1.038</v>
+        <v>0.989</v>
       </c>
       <c r="E16" t="n">
-        <v>-2.3</v>
+        <v>3.6</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.3</v>
+        <v>2.5</v>
       </c>
       <c r="G16" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1273,19 +1273,19 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>18174</v>
+        <v>203013</v>
       </c>
       <c r="K16" t="n">
-        <v>13478</v>
+        <v>229936</v>
       </c>
       <c r="L16" t="n">
-        <v>29.79</v>
+        <v>5.12</v>
       </c>
       <c r="M16" t="n">
-        <v>30.99</v>
+        <v>5.01</v>
       </c>
       <c r="N16" t="n">
-        <v>4</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
MPCC Q2 refresh REGEN: NAV 2.05->2.10 INSIDE the prereg band [1.90,2.30] (predicted 2.09-2.12), EV -27.5->-24.8pp, TRIM/SHORT + POSITION_UNRELIABLE stand, forward invariance 0.0 on 24 names; gate 25 rows / 0 UNEXPLAINED / 1 explained (MPCC row annotated in-log, rides the next owner ratify); 14 of 25 names at Q2 vintage
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -1251,16 +1251,16 @@
         <v>1.04</v>
       </c>
       <c r="D16" t="n">
-        <v>1.2</v>
+        <v>1.193</v>
       </c>
       <c r="E16" t="n">
-        <v>-27.5</v>
+        <v>-24.8</v>
       </c>
       <c r="F16" t="n">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="G16" t="n">
-        <v>-8.4</v>
+        <v>-7.1</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1273,19 +1273,19 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>214794</v>
+        <v>192190</v>
       </c>
       <c r="K16" t="n">
-        <v>60526</v>
+        <v>54836</v>
       </c>
       <c r="L16" t="n">
-        <v>2.07</v>
+        <v>2.15</v>
       </c>
       <c r="M16" t="n">
-        <v>2.62</v>
+        <v>2.65</v>
       </c>
       <c r="N16" t="n">
-        <v>19.2</v>
+        <v>17.7</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Refresh-consequent test re-pins (dated; the FLNG/TRMD pins-advance-WITH-the-pair convention) + guard completions: BWLP pins to the Q2 sheet (debt 814.2/leases 118.4/NCI 216.3), MPCC baseline 2.10-band, FRO fixture Q2 (counts 42/19/18, ramp 40, un-anchored implied ~1.51 re-pinned, warning fixture Q2/44.19), NAT dividend-window + suezmax-recal fixtures Q2, HAFN scenario band 5.59±5% (JV correction + ten-hull legs), quarter-coherence lagging specimen FRO->CMBT (deferred 9/03); HAFN registered in newbuild_specs (scrubber=false conservative, no NB statement — SB/ECO rule), hafn [ESTIMATE] floor marker restored (xfail-strict queue intact), hafn on_curve_total cross-foot 100, MPCC provenance phrasing cited; all five family sidecars re-run after the FV-moving pairs
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -887,16 +887,16 @@
         <v>0.85</v>
       </c>
       <c r="D9" t="n">
-        <v>2.325</v>
+        <v>2.398</v>
       </c>
       <c r="E9" t="n">
-        <v>-54.7</v>
+        <v>-55.8</v>
       </c>
       <c r="F9" t="n">
-        <v>-21.6</v>
+        <v>-22.2</v>
       </c>
       <c r="G9" t="n">
-        <v>11.4</v>
+        <v>11.3</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -909,19 +909,19 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>667460</v>
+        <v>678594</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>3.07</v>
+        <v>3</v>
       </c>
       <c r="M9" t="n">
-        <v>7.54</v>
+        <v>7.53</v>
       </c>
       <c r="N9" t="n">
-        <v>66.09999999999999</v>
+        <v>67.09999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -991,16 +991,16 @@
         <v>1.03</v>
       </c>
       <c r="D11" t="n">
-        <v>1.404</v>
+        <v>1.554</v>
       </c>
       <c r="E11" t="n">
-        <v>-22.6</v>
+        <v>-34</v>
       </c>
       <c r="F11" t="n">
-        <v>-8.1</v>
+        <v>-14.2</v>
       </c>
       <c r="G11" t="n">
-        <v>6.4</v>
+        <v>5.7</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1013,19 +1013,19 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>126841</v>
+        <v>159436</v>
       </c>
       <c r="K11" t="n">
-        <v>52720</v>
+        <v>53122</v>
       </c>
       <c r="L11" t="n">
-        <v>6.56</v>
+        <v>5.59</v>
       </c>
       <c r="M11" t="n">
-        <v>9.02</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>29</v>
+        <v>39.7</v>
       </c>
     </row>
     <row r="12">
@@ -1511,16 +1511,16 @@
         <v>1.33</v>
       </c>
       <c r="D21" t="n">
-        <v>1.208</v>
+        <v>1.196</v>
       </c>
       <c r="E21" t="n">
-        <v>-37.1</v>
+        <v>-36</v>
       </c>
       <c r="F21" t="n">
-        <v>-29.1</v>
+        <v>-28.6</v>
       </c>
       <c r="G21" t="n">
-        <v>-21</v>
+        <v>-21.3</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1533,19 +1533,19 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>682553</v>
+        <v>715733</v>
       </c>
       <c r="K21" t="n">
-        <v>465663</v>
+        <v>499366</v>
       </c>
       <c r="L21" t="n">
-        <v>27.79</v>
+        <v>28.29</v>
       </c>
       <c r="M21" t="n">
-        <v>34.92</v>
+        <v>34.78</v>
       </c>
       <c r="N21" t="n">
-        <v>16.1</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="22">
@@ -1719,16 +1719,16 @@
         <v>1.27</v>
       </c>
       <c r="D25" t="n">
-        <v>1.156</v>
+        <v>1.157</v>
       </c>
       <c r="E25" t="n">
-        <v>-39.9</v>
+        <v>-39.6</v>
       </c>
       <c r="F25" t="n">
-        <v>-34.4</v>
+        <v>-34.3</v>
       </c>
       <c r="G25" t="n">
-        <v>-29</v>
+        <v>-28.9</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1741,19 +1741,19 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>253816</v>
+        <v>252777</v>
       </c>
       <c r="K25" t="n">
-        <v>188145</v>
+        <v>187737</v>
       </c>
       <c r="L25" t="n">
-        <v>14.46</v>
+        <v>14.52</v>
       </c>
       <c r="M25" t="n">
-        <v>17.07</v>
+        <v>17.1</v>
       </c>
       <c r="N25" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="26">

</xml_diff>

<commit_message>
CAPT H1 refresh REGEN + HALT-INVESTIGATION RESOLVED: NAV 15.48->17.32 landed 0.02 (0.1%) ABOVE the frozen band [14.70,17.30] — decomposed and ACCEPTED (the June 3-contract acquisition contributes +1.71/sh at curve marks: bought at locked 2025 contract ~65M/hull below the war-market age-0 level; the prereg's neutral-if-at-market assumption was the miss, not an input error; issuer's own 8/18 option appraisals corroborate direction). CONDITION 5 ENFORCED: HOLD->BUY flip recorded-NOT-actionable, POSITION_UNRELIABLE + GOVERNED-WIDE stand, no void retires outside R4; crude sidecar re-run (CAPT WEIGHT-DRIVEN: +6.7% BUY Set A <-> -21.2% TRIM conservative brackets); k 1.26->1.17; gate 25 rows / 0 UNEXPLAINED / 1 explained; SANITY OK -22.4%; Stage-B VLCC TC 97,076 captured; provenance citations tightened; 20 of 25 names at Q2 vintage
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/broker_nav_sweep.xlsx
+++ b/outputs/broker_nav_sweep.xlsx
@@ -627,20 +627,20 @@
         <v>0.72</v>
       </c>
       <c r="D4" t="n">
-        <v>1.263</v>
+        <v>1.175</v>
       </c>
       <c r="E4" t="n">
-        <v>-2.7</v>
+        <v>6.7</v>
       </c>
       <c r="F4" t="n">
-        <v>18.1</v>
+        <v>22.3</v>
       </c>
       <c r="G4" t="n">
-        <v>38.9</v>
+        <v>37.8</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>HOLD (fairly valued)</t>
+          <t>BUY (undervalued)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -649,19 +649,19 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>207425</v>
+        <v>63532</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>16.02</v>
+        <v>17.56</v>
       </c>
       <c r="M4" t="n">
-        <v>22.86</v>
+        <v>22.69</v>
       </c>
       <c r="N4" t="n">
-        <v>41.5</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="5">

</xml_diff>